<commit_message>
Including drop in components for Rev3
</commit_message>
<xml_diff>
--- a/Charge_Indicator/BOM and Order Sheet/Cost Tracking Redact/Cost_Tracking_Sheet.xlsx
+++ b/Charge_Indicator/BOM and Order Sheet/Cost Tracking Redact/Cost_Tracking_Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nathanfikes/Documents/GitHub/AutoNav-Charge_Indicator-KiCad_Pcb/Charge_Indicator/BOM and Order Sheet/Cost Tracking Redact/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08733B0B-1FDA-0548-8B34-C6B49E5C3194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10F11A3-9759-A244-B90B-E3220A54BEA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="3840" windowWidth="29880" windowHeight="14700" xr2:uid="{F977D430-13CE-AD47-96E5-85BBB755CDD5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t>Supplier</t>
   </si>
@@ -92,18 +92,18 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -111,13 +111,13 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="游ゴシック"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="6"/>
-      <name val="游ゴシック"/>
+      <name val="Aptos Narrow"/>
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
@@ -194,14 +194,14 @@
     <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="通貨 [0.00]" xfId="1" builtinId="4"/>
-    <cellStyle name="標準" xfId="0" builtinId="0"/>
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -222,7 +222,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -539,16 +539,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5429AA39-1145-AF43-8726-DB045179E867}">
   <dimension ref="A3:M46"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="23" customWidth="1"/>
-    <col min="13" max="13" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="133" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" ht="16" customHeight="1">
+    <row r="3" spans="1:3" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -559,7 +559,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
@@ -570,7 +570,7 @@
         <v>22.43</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="5">
         <v>118559797</v>
       </c>
@@ -581,7 +581,7 @@
         <v>116.94</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="5">
         <v>119203286</v>
       </c>
@@ -592,7 +592,7 @@
         <v>11.23</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -603,7 +603,7 @@
         <v>31.65</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -614,7 +614,7 @@
         <v>5.24</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -625,7 +625,7 @@
         <v>18.690000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -636,66 +636,72 @@
         <v>15.76</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="10">
         <v>5.23</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="7"/>
-    </row>
-    <row r="13" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="5">
+        <v>98147822</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="10">
+        <v>8.08</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="4"/>
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="4"/>
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="4"/>
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="4"/>
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="2:3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="6">
         <f>SUM(C4:C16)</f>
-        <v>227.17</v>
-      </c>
-    </row>
-    <row r="45" spans="5:13">
+        <v>235.25</v>
+      </c>
+    </row>
+    <row r="45" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
       <c r="H45" s="3"/>
-      <c r="L45" s="10"/>
-      <c r="M45" s="10"/>
-    </row>
-    <row r="46" spans="5:13">
+      <c r="L45" s="11"/>
+      <c r="M45" s="11"/>
+    </row>
+    <row r="46" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E46" s="2"/>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
       <c r="H46" s="3"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="10"/>
+      <c r="L46" s="11"/>
+      <c r="M46" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>